<commit_message>
Actualizar los estados del backlog con los PR #38 y #39
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/RecyTrack_Product_Backlog.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/RecyTrack_Product_Backlog.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$K$51</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr fullCalcOnLoad="1" iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -1708,14 +1708,18 @@
       <c r="H10" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>45</v>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J10" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K10" s="6" t="s">
-        <v>47</v>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Base del resto del sprint. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1778,13 +1782,19 @@
       <c r="H12" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="I12" s="7" t="s">
-        <v>45</v>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J12" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K12" s="6"/>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio y reglas de áreas en main (PR #38, #39); falta la pantalla del panel (#33).</t>
+        </is>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
@@ -1846,14 +1856,18 @@
       <c r="H14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="I14" s="7" t="s">
-        <v>45</v>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J14" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K14" s="6" t="s">
-        <v>65</v>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se adelantó desde S5. Regla para cambiar de área en main (PR #39); falta la pantalla del panel (#33).</t>
+        </is>
       </c>
     </row>
     <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1881,14 +1895,18 @@
       <c r="H15" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>45</v>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J15" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="K15" s="6" t="s">
-        <v>70</v>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se adelantó desde S3. No se usan códigos para el validador. Regla para nombrar al validador en main (PR #39); falta el selector en el panel (#33).</t>
+        </is>
       </c>
     </row>
     <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1951,14 +1969,18 @@
       <c r="H17" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I17" s="7" t="s">
-        <v>79</v>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J17" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K17" s="6" t="s">
-        <v>80</v>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Unión al área con reglas en main (PR #38, #39); falta mostrar el nombre del área antes de confirmar (#29).</t>
+        </is>
       </c>
     </row>
     <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1986,13 +2008,19 @@
       <c r="H18" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>79</v>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J18" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="6"/>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
@@ -2019,13 +2047,19 @@
       <c r="H19" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>87</v>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J19" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="6"/>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
@@ -2052,14 +2086,18 @@
       <c r="H20" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I20" s="7" t="s">
-        <v>79</v>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J20" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K20" s="6" t="s">
-        <v>91</v>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. El contenedor ya se valida contra la planta. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
       </c>
     </row>
     <row r="21" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2087,13 +2125,19 @@
       <c r="H21" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>87</v>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J21" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="6"/>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
@@ -2120,13 +2164,19 @@
       <c r="H22" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I22" s="7" t="s">
-        <v>87</v>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J22" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="K22" s="6"/>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
@@ -2256,13 +2306,19 @@
       <c r="H26" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I26" s="7" t="s">
-        <v>87</v>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J26" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="K26" s="6"/>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Servicio y reglas del retiro en main (PR #38, #39); falta la pantalla del panel (#35).</t>
+        </is>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
@@ -2289,14 +2345,18 @@
       <c r="H27" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I27" s="7" t="s">
-        <v>87</v>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J27" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="K27" s="6" t="s">
-        <v>120</v>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El gestor estaba en la propuesta inicial a la viña. Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
       </c>
     </row>
     <row r="28" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2324,14 +2384,18 @@
       <c r="H28" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I28" s="7" t="s">
-        <v>79</v>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J28" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="K28" s="6" t="s">
-        <v>126</v>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. El certificado ya incluye el área. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
       </c>
     </row>
     <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2359,14 +2423,18 @@
       <c r="H29" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>79</v>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J29" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="K29" s="6" t="s">
-        <v>130</v>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Reporte adaptado a planta y áreas (PR #38); falta la participación por área en el PDF y el botón del panel (#35).</t>
+        </is>
       </c>
     </row>
     <row r="30" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2464,13 +2532,19 @@
       <c r="H32" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I32" s="7" t="s">
-        <v>87</v>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J32" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K32" s="6"/>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. El retiro cierra las incidencias en el mismo lote (PR #38, #39); falta la pantalla del retiro (#35).</t>
+        </is>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
@@ -2530,13 +2604,19 @@
       <c r="H34" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I34" s="7" t="s">
-        <v>79</v>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J34" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K34" s="6"/>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
@@ -2563,14 +2643,18 @@
       <c r="H35" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="I35" s="7" t="s">
-        <v>79</v>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J35" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="K35" s="6" t="s">
-        <v>156</v>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Ranking por participación de áreas en main (PR #38); falta el rediseño (#30).</t>
+        </is>
       </c>
     </row>
     <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2598,13 +2682,19 @@
       <c r="H36" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="I36" s="7" t="s">
-        <v>87</v>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J36" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="K36" s="6"/>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Servicio y reglas de la campaña en main (PR #38, #39); falta la sección Incentivo del panel (#34).</t>
+        </is>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
@@ -2936,13 +3026,19 @@
       <c r="H46" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="I46" s="7" t="s">
-        <v>87</v>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="J46" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K46" s="6"/>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+        </is>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">

</xml_diff>

<commit_message>
Actualizar el Product Backlog al cierre del S2
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/RecyTrack_Product_Backlog.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/RecyTrack_Product_Backlog.xlsx
@@ -1475,8 +1475,10 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ordenado por sprint y prioridad. Estado al 18 de octubre de 2026. Las columnas Prioridad, Puntos, Sprint y Estado son editables.</t>
+        </is>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1705,12 +1707,14 @@
       <c r="G10" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H10" s="7" t="s">
-        <v>44</v>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J10" s="6" t="s">
@@ -1718,7 +1722,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Base del resto del sprint. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #38, aprobado por Álvaro, y PR #39, aprobado por Vicente).</t>
         </is>
       </c>
     </row>
@@ -1744,17 +1748,23 @@
       <c r="G11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>45</v>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J11" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K11" s="6" t="s">
-        <v>53</v>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #43, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1779,12 +1789,14 @@
       <c r="G12" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="7" t="s">
-        <v>44</v>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J12" s="6" t="s">
@@ -1792,7 +1804,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Servicio y reglas de áreas en main (PR #38, #39); falta la pantalla del panel (#33).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #44, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -1818,17 +1830,23 @@
       <c r="G13" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>45</v>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J13" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K13" s="6" t="s">
-        <v>61</v>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #44, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1853,12 +1871,14 @@
       <c r="G14" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="7" t="s">
-        <v>44</v>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J14" s="6" t="s">
@@ -1866,7 +1886,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Se adelantó desde S5. Regla para cambiar de área en main (PR #39); falta la pantalla del panel (#33).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #44, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -1892,12 +1912,14 @@
       <c r="G15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H15" s="7" t="s">
-        <v>44</v>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J15" s="6" t="s">
@@ -1905,7 +1927,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Se adelantó desde S3. No se usan códigos para el validador. Regla para nombrar al validador en main (PR #39); falta el selector en el panel (#33).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #44, fusionado por el administrador sin aprobación de otro integrante). No se usan códigos para el validador.</t>
         </is>
       </c>
     </row>
@@ -1931,17 +1953,23 @@
       <c r="G16" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>45</v>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J16" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="K16" s="6" t="s">
-        <v>74</v>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #44, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1966,12 +1994,14 @@
       <c r="G17" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H17" s="7" t="s">
-        <v>78</v>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J17" s="6" t="s">
@@ -1979,7 +2009,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Unión al área con reglas en main (PR #38, #39); falta mostrar el nombre del área antes de confirmar (#29).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante). Muestra el nombre del área antes de unirse.</t>
         </is>
       </c>
     </row>
@@ -2005,12 +2035,14 @@
       <c r="G18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="7" t="s">
-        <v>78</v>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J18" s="6" t="s">
@@ -2018,7 +2050,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #38, aprobado por Álvaro, y PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -2044,12 +2076,14 @@
       <c r="G19" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H19" s="7" t="s">
-        <v>78</v>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J19" s="6" t="s">
@@ -2057,7 +2091,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #38, aprobado por Álvaro).</t>
         </is>
       </c>
     </row>
@@ -2083,12 +2117,14 @@
       <c r="G20" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H20" s="7" t="s">
-        <v>78</v>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J20" s="6" t="s">
@@ -2096,7 +2132,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. El contenedor ya se valida contra la planta. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #39, aprobado por Vicente). El contenedor se valida contra la planta.</t>
         </is>
       </c>
     </row>
@@ -2122,12 +2158,14 @@
       <c r="G21" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H21" s="7" t="s">
-        <v>78</v>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J21" s="6" t="s">
@@ -2135,7 +2173,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #38, aprobado por Álvaro).</t>
         </is>
       </c>
     </row>
@@ -2161,12 +2199,14 @@
       <c r="G22" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H22" s="7" t="s">
-        <v>78</v>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J22" s="6" t="s">
@@ -2174,7 +2214,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #39, aprobado por Vicente).</t>
         </is>
       </c>
     </row>
@@ -2200,17 +2240,23 @@
       <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H23" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>79</v>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J23" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="K23" s="6" t="s">
-        <v>102</v>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="24" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2235,17 +2281,23 @@
       <c r="G24" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H24" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>79</v>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J24" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="K24" s="6" t="s">
-        <v>106</v>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2270,16 +2322,24 @@
       <c r="G25" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H25" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>87</v>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J25" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="K25" s="6"/>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
@@ -2303,12 +2363,14 @@
       <c r="G26" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H26" s="7" t="s">
-        <v>114</v>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J26" s="6" t="s">
@@ -2316,7 +2378,7 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Servicio y reglas del retiro en main (PR #38, #39); falta la pantalla del panel (#35).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #46 y #47, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -2342,12 +2404,14 @@
       <c r="G27" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H27" s="7" t="s">
-        <v>114</v>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J27" s="6" t="s">
@@ -2355,7 +2419,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">El gestor estaba en la propuesta inicial a la viña. Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #38, aprobado por Álvaro, y PR #39, aprobado por Vicente).</t>
         </is>
       </c>
     </row>
@@ -2381,12 +2445,14 @@
       <c r="G28" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H28" s="7" t="s">
-        <v>114</v>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J28" s="6" t="s">
@@ -2394,7 +2460,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. El certificado ya incluye el área. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #38, aprobado por Álvaro). El certificado incluye el área.</t>
         </is>
       </c>
     </row>
@@ -2420,12 +2486,14 @@
       <c r="G29" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H29" s="7" t="s">
-        <v>114</v>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J29" s="6" t="s">
@@ -2433,7 +2501,7 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Reporte adaptado a planta y áreas (PR #38); falta la participación por área en el PDF y el botón del panel (#35).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #46, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -2462,14 +2530,18 @@
       <c r="H30" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I30" s="7" t="s">
-        <v>87</v>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente</t>
+        </is>
       </c>
       <c r="J30" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K30" s="6" t="s">
-        <v>135</v>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente para antes del piloto (#36).</t>
+        </is>
       </c>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2497,14 +2569,18 @@
       <c r="H31" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I31" s="7" t="s">
-        <v>87</v>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente</t>
+        </is>
       </c>
       <c r="J31" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K31" s="6" t="s">
-        <v>139</v>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Depende de los datos que entregue la viña (#36).</t>
+        </is>
       </c>
     </row>
     <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2529,12 +2605,14 @@
       <c r="G32" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H32" s="7" t="s">
-        <v>114</v>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J32" s="6" t="s">
@@ -2542,7 +2620,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. El retiro cierra las incidencias en el mismo lote (PR #38, #39); falta la pantalla del retiro (#35).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #46, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -2568,16 +2646,24 @@
       <c r="G33" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="I33" s="7" t="s">
-        <v>87</v>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J33" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="K33" s="6"/>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #46, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
@@ -2601,12 +2687,14 @@
       <c r="G34" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H34" s="7" t="s">
-        <v>114</v>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J34" s="6" t="s">
@@ -2614,7 +2702,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -2640,12 +2728,14 @@
       <c r="G35" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H35" s="7" t="s">
-        <v>154</v>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J35" s="6" t="s">
@@ -2653,7 +2743,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Ranking por participación de áreas en main (PR #38); falta el rediseño (#30).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -2679,12 +2769,14 @@
       <c r="G36" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H36" s="7" t="s">
-        <v>154</v>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J36" s="6" t="s">
@@ -2692,7 +2784,7 @@
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Servicio y reglas de la campaña en main (PR #38, #39); falta la sección Incentivo del panel (#34).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #45, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -2718,16 +2810,24 @@
       <c r="G37" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H37" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="I37" s="7" t="s">
-        <v>87</v>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J37" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K37" s="6"/>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #43 y #49, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
@@ -2751,16 +2851,24 @@
       <c r="G38" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H38" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>87</v>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J38" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K38" s="6"/>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
@@ -2784,17 +2892,23 @@
       <c r="G39" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H39" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>87</v>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J39" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K39" s="6" t="s">
-        <v>169</v>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #45, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2819,17 +2933,23 @@
       <c r="G40" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H40" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="I40" s="7" t="s">
-        <v>79</v>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J40" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="K40" s="6" t="s">
-        <v>175</v>
+      <c r="K40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="41" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2854,17 +2974,23 @@
       <c r="G41" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H41" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="I41" s="7" t="s">
-        <v>87</v>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J41" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K41" s="6" t="s">
-        <v>179</v>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #43, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="42" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2955,16 +3081,24 @@
       <c r="G44" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H44" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="I44" s="7" t="s">
-        <v>87</v>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J44" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K44" s="6"/>
+      <c r="K44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #46, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
@@ -2988,17 +3122,23 @@
       <c r="G45" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H45" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="I45" s="7" t="s">
-        <v>79</v>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
       </c>
       <c r="J45" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="K45" s="6" t="s">
-        <v>196</v>
+      <c r="K45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada en el S2 (PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
+        </is>
       </c>
     </row>
     <row r="46" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3023,12 +3163,14 @@
       <c r="G46" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H46" s="7" t="s">
-        <v>183</v>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
+          <t xml:space="preserve">Hecho</t>
         </is>
       </c>
       <c r="J46" s="6" t="s">
@@ -3036,7 +3178,7 @@
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adelantada al S2. Código y reglas en main (PR #38, #39); falta publicar y probar en teléfono (#36).</t>
+          <t xml:space="preserve">Terminada en el S2 (PR #38, aprobado por Álvaro; PR #39, aprobado por Vicente; y PR #42, fusionado por el administrador sin aprobación de otro integrante).</t>
         </is>
       </c>
     </row>
@@ -3065,13 +3207,19 @@
       <c r="H47" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="I47" s="7" t="s">
-        <v>87</v>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente</t>
+        </is>
       </c>
       <c r="J47" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="K47" s="6"/>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estaba en el issue #30, pero no se implementó.</t>
+        </is>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">

</xml_diff>